<commit_message>
Validated time environment and virtual hardware for manual mode.
</commit_message>
<xml_diff>
--- a/src/rattlesnake/examples/environment/time/time_v3.xlsx
+++ b/src/rattlesnake/examples/environment/time/time_v3.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\examples\environment\time\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmlangs\Desktop\rattlesnake-vibration-controller-headless\src\rattlesnake\examples\environment\time\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1087A690-A54E-451D-8953-6DCEF1B943CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{878C84BD-2E0E-43DB-8A2A-D486F810C93E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6070" yWindow="1960" windowWidth="28790" windowHeight="15350" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="19110" yWindow="0" windowWidth="19380" windowHeight="20970" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Time 0" sheetId="3" r:id="rId1"/>
@@ -537,27 +537,27 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A7">
-        <v>5</v>
+        <v>6.5</v>
       </c>
       <c r="B7" t="s">
         <v>0</v>
       </c>
       <c r="C7" t="s">
-        <v>17</v>
-      </c>
-      <c r="D7">
-        <v>5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8" t="s">
+        <v>0</v>
+      </c>
+      <c r="C8" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8">
         <v>5</v>
-      </c>
-      <c r="B8" t="s">
-        <v>0</v>
-      </c>
-      <c r="C8" t="s">
-        <v>14</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.35">

</xml_diff>